<commit_message>
Fixes to notebooks 06b, 07 and 08
</commit_message>
<xml_diff>
--- a/notebooks/qgis_lab_08/debris_flow_measurements.xlsx
+++ b/notebooks/qgis_lab_08/debris_flow_measurements.xlsx
@@ -1,66 +1,123 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Python\silesia-slopes\notebooks\qgis_lab_08\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3324850-C3E9-4EA9-8E87-FC43081632FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="measurements" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="measurements" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>Skamsdalen debris-flow measurements — fill in as you digitise in QGIS</t>
+  </si>
+  <si>
+    <t>Read elevations on the fly with the Identify Features tool on the DTM; read distances off the Measure Line tool. Type values straight into the white cells. H and beta (grey) are computed automatically as a sanity check — leave them alone.</t>
+  </si>
+  <si>
+    <t>flow_id</t>
+  </si>
+  <si>
+    <t>z_source</t>
+  </si>
+  <si>
+    <t>z_beta</t>
+  </si>
+  <si>
+    <t>z_toe</t>
+  </si>
+  <si>
+    <t>L_beta</t>
+  </si>
+  <si>
+    <t>L_obs</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>beta_deg</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="13"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
+      <i/>
       <sz val="9"/>
+      <color rgb="FF555555"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
+        <fgColor rgb="FF2F5597"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8E8E8"/>
+        <fgColor rgb="FFE8E8E8"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,109 +131,52 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="FFBBBBBB"/>
       </left>
       <right style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="FFBBBBBB"/>
       </right>
       <top style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="FFBBBBBB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="FFBBBBBB"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -464,166 +464,189 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col min="1" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Skamsdalen debris-flow measurements — fill in as you digitise in QGIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Read elevations on the fly with the Identify Features tool on the DTM; read distances off the Measure Line tool. Type values straight into the white cells. H and beta (grey) are computed automatically as a sanity check — leave them alone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>flow_id</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>z_source</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>z_beta</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>z_toe</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>L_beta</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>L_obs</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>beta_deg</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
+    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+    </row>
+    <row r="2" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6">
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1060</v>
+      </c>
+      <c r="C5" s="3">
+        <v>924</v>
+      </c>
+      <c r="D5" s="3">
+        <v>892</v>
+      </c>
+      <c r="E5" s="3">
+        <v>370</v>
+      </c>
+      <c r="F5" s="3">
+        <v>570</v>
+      </c>
+      <c r="G5" s="4">
         <f>IF(AND(B5&lt;&gt;"",D5&lt;&gt;""),B5-D5,"")</f>
-        <v/>
-      </c>
-      <c r="H5" s="6">
+        <v>168</v>
+      </c>
+      <c r="H5" s="4">
         <f>IF(AND(B5&lt;&gt;"",C5&lt;&gt;"",E5&lt;&gt;""),DEGREES(ATAN((B5-C5)/E5)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+        <v>20.181790699981697</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6">
+      <c r="B6" s="3">
+        <v>1094</v>
+      </c>
+      <c r="C6" s="3">
+        <v>925</v>
+      </c>
+      <c r="D6" s="3">
+        <v>892</v>
+      </c>
+      <c r="E6" s="3">
+        <v>391</v>
+      </c>
+      <c r="F6" s="3">
+        <v>675</v>
+      </c>
+      <c r="G6" s="4">
         <f>IF(AND(B6&lt;&gt;"",D6&lt;&gt;""),B6-D6,"")</f>
-        <v/>
-      </c>
-      <c r="H6" s="6">
+        <v>202</v>
+      </c>
+      <c r="H6" s="4">
         <f>IF(AND(B6&lt;&gt;"",C6&lt;&gt;"",E6&lt;&gt;""),DEGREES(ATAN((B6-C6)/E6)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
+        <v>23.37521072952228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="6">
+      <c r="B7" s="3">
+        <v>1085</v>
+      </c>
+      <c r="C7" s="3">
+        <v>934</v>
+      </c>
+      <c r="D7" s="3">
+        <v>894</v>
+      </c>
+      <c r="E7" s="3">
+        <v>407</v>
+      </c>
+      <c r="F7" s="3">
+        <v>627</v>
+      </c>
+      <c r="G7" s="4">
         <f>IF(AND(B7&lt;&gt;"",D7&lt;&gt;""),B7-D7,"")</f>
-        <v/>
-      </c>
-      <c r="H7" s="6">
+        <v>191</v>
+      </c>
+      <c r="H7" s="4">
         <f>IF(AND(B7&lt;&gt;"",C7&lt;&gt;"",E7&lt;&gt;""),DEGREES(ATAN((B7-C7)/E7)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+        <v>20.355225029891734</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="6">
+      <c r="B8" s="3">
+        <v>1150</v>
+      </c>
+      <c r="C8" s="3">
+        <v>927</v>
+      </c>
+      <c r="D8" s="3">
+        <v>909</v>
+      </c>
+      <c r="E8" s="3">
+        <v>553</v>
+      </c>
+      <c r="F8" s="3">
+        <v>703</v>
+      </c>
+      <c r="G8" s="4">
         <f>IF(AND(B8&lt;&gt;"",D8&lt;&gt;""),B8-D8,"")</f>
-        <v/>
-      </c>
-      <c r="H8" s="6">
+        <v>241</v>
+      </c>
+      <c r="H8" s="4">
         <f>IF(AND(B8&lt;&gt;"",C8&lt;&gt;"",E8&lt;&gt;""),DEGREES(ATAN((B8-C8)/E8)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
+        <v>21.962001409512215</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="6">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="4" t="str">
         <f>IF(AND(B9&lt;&gt;"",D9&lt;&gt;""),B9-D9,"")</f>
         <v/>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="4" t="str">
         <f>IF(AND(B9&lt;&gt;"",C9&lt;&gt;"",E9&lt;&gt;""),DEGREES(ATAN((B9-C9)/E9)),"")</f>
         <v/>
       </c>

</xml_diff>